<commit_message>
Doku , Spec Update curent status
</commit_message>
<xml_diff>
--- a/docs/nova_overview.xlsx
+++ b/docs/nova_overview.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stefan_pro/fleet/docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stefan_pro/Documents/Claude/Projects/nova/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCC8F0C6-5236-8147-A47D-788BB2AE5A91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{995A1D40-8484-B049-BD0F-3C97B332781B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="25600" xr2:uid="{189BD8D0-FCFC-8748-8061-DE49C9010CB9}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="38400" windowHeight="24980" xr2:uid="{189BD8D0-FCFC-8748-8061-DE49C9010CB9}"/>
   </bookViews>
   <sheets>
-    <sheet name="V1" sheetId="2" r:id="rId1"/>
-    <sheet name="V0" sheetId="1" r:id="rId2"/>
+    <sheet name="V2_26_04_30" sheetId="3" r:id="rId1"/>
+    <sheet name="V1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">V0!$A$2:$C$26</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'V1'!$A$2:$C$26</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'V1'!$A$2:$C$26</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">V2_26_04_30!$A$2:$C$28</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="103">
   <si>
     <t>Zielsetzung</t>
   </si>
@@ -85,11 +85,6 @@
     <t>Zentral auf DEV-Node</t>
   </si>
   <si>
-    <t>Node:
-- zsh Login Profile für novaadm setzen
-- Runtime Software über bundle brew aktualisieren</t>
-  </si>
-  <si>
     <t>Tasks</t>
   </si>
   <si>
@@ -136,10 +131,6 @@
   </si>
   <si>
     <t xml:space="preserve">Security </t>
-  </si>
-  <si>
-    <t>SSH Keys lokal
-keine Secrets in Repo</t>
   </si>
   <si>
     <r>
@@ -177,12 +168,6 @@
     </r>
   </si>
   <si>
-    <t>Node:
-- git pull
-- 00_init_novaadm.sh
-- 15_init_runtime.sh</t>
-  </si>
-  <si>
     <t>nova-uat , nova-prod</t>
   </si>
   <si>
@@ -195,19 +180,6 @@
     <t>~/&lt;repo&gt;</t>
   </si>
   <si>
-    <t>DEV-Node:
-- ./dotfiles/zsh/.zshrc – modify
-- ./dotfiles/zsh/.p10k.zsh – modify
-- 05_set_node_name.sh – modify
-- 10_seed_node.sh – run
-- 12_seed_ssh.sh – run
-New Node:
-- 05_set_node_name.sh – modify
-- Technischen User novaadm anlegen
-- ssh Konfiguration
-- git clone github.com:&lt;gituser&gt;/&lt;repo&gt;.git</t>
-  </si>
-  <si>
     <t>Spezifikation Zielsystem</t>
   </si>
   <si>
@@ -221,11 +193,6 @@
   </si>
   <si>
     <t>Node in Environment (1:1 Beziehung)</t>
-  </si>
-  <si>
-    <t>Neuer Mac als Environment in NovaPlatform als nova-&lt;Environment&gt; vorbereitet
-- Netzwerk konfiguriert
-- Repository auf New Node geclont</t>
   </si>
   <si>
     <t>Environment</t>
@@ -287,12 +254,188 @@
 UAT-Rot.
 Die Umgebung wird im Prompt dargestellt.</t>
   </si>
+  <si>
+    <t>Job Development und Execution Plattform für MacOS Cluster.
+Zentaler Hub mit Worker Nodes</t>
+  </si>
+  <si>
+    <t>Hub-Node</t>
+  </si>
+  <si>
+    <t>nova-hub</t>
+  </si>
+  <si>
+    <t>Deployment SW auf Worker Nodes. Job Control Worker Nodes</t>
+  </si>
+  <si>
+    <t>nova-w&lt;1..n&gt;</t>
+  </si>
+  <si>
+    <t>Worker Node: Host und Worker Nummer</t>
+  </si>
+  <si>
+    <t>git Repository nova</t>
+  </si>
+  <si>
+    <t>https://github.com/gershu/nova</t>
+  </si>
+  <si>
+    <t>~/Documents/Claude/Projects/nova</t>
+  </si>
+  <si>
+    <t>nova-hub: node deployment - JobControl</t>
+  </si>
+  <si>
+    <t>ssh nova-2 ~/nova/scripts/node_deploy.sh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Node Spezifikation </t>
+  </si>
+  <si>
+    <t>Rolle, Specs</t>
+  </si>
+  <si>
+    <t>Über git pull , Requirements in Skript</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ~/nova/scripts/nova_submit.sh hello_world nova-w2
+~/nova/scripts/node_status.sh
+ ~/nova/scripts/cluster_status.sh</t>
+  </si>
+  <si>
+    <t>config/nodes.yaml
+ nova-w1:
+    role: worker
+    chip: arm64
+    ram_gb: 16
+    os: macos-15
+    notes: "MacbookPro M1 Apple Silicon, Editor und Worker"</t>
+  </si>
+  <si>
+    <t>Workload Repos</t>
+  </si>
+  <si>
+    <t>jedes Repo wird unter ~/&lt;lokales-verzeichnis&gt;
+auf jedem Node geklont</t>
+  </si>
+  <si>
+    <t>~/csp_scanner</t>
+  </si>
+  <si>
+    <t>Worker Node</t>
+  </si>
+  <si>
+    <t>Führt Task / Wokload aus</t>
+  </si>
+  <si>
+    <t>Workload</t>
+  </si>
+  <si>
+    <t>Eigenes Repo mit universellem Start Script</t>
+  </si>
+  <si>
+    <t>Role</t>
+  </si>
+  <si>
+    <t>Zentrales Hub, Worker</t>
+  </si>
+  <si>
+    <t>Neuen Mac als Worker Node definieren
+- Metadaten in config/nodes.yaml ergänzrn
+-  Technical User novaadm anlegen
+- Hostnamen setzen
+- ssh Keys bereitstellen
+- Initiales Bootstrapping</t>
+  </si>
+  <si>
+    <t>nova-w4</t>
+  </si>
+  <si>
+    <t>Node:
+- git pull aktuelle Sourcen
+- apply changes : Dot Files
+- bundle brew Software Installation und Update
+- Für Hub Picker Start</t>
+  </si>
+  <si>
+    <t>job picker</t>
+  </si>
+  <si>
+    <t>Dämon auf Hub, alle 10sek. Startet Workload &lt;~workload&gt; auf Worker Node &lt;i&gt;  mit parameter &lt;para.json&gt;</t>
+  </si>
+  <si>
+    <t>cat &gt; ~/jobs_test.json &lt;&lt;'EOF'
+{"ticker": "AAPL", "horizon_days": 30}
+EOF
+JOB2=$(~/nova/scripts/nova_submit.sh hello_world nova-w1 )
+echo "Submitted: $JOB2"</t>
+  </si>
+  <si>
+    <t>Starte Workload auf Hub</t>
+  </si>
+  <si>
+    <t>nova_submit.sh hello_world nova-w1</t>
+  </si>
+  <si>
+    <t>Stock Scanner</t>
+  </si>
+  <si>
+    <t>Spezifikation Nova Plattform</t>
+  </si>
+  <si>
+    <t>Aktueller Stand</t>
+  </si>
+  <si>
+    <t>ok</t>
+  </si>
+  <si>
+    <t>Neu : Hub soll auch Job ausführen können</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neu: Universeller Parser für JSON-Parameter </t>
+  </si>
+  <si>
+    <t>Neu: 
+- Return Wert Logfile Name
+- Verarbeitung im Hintergrund / parallel</t>
+  </si>
+  <si>
+    <t>Deployment Node</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ggfs: Split 
+- Profile für Terminal separt handlen
+- angepasste SW Build für ältere OS Version
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MacbookPro , StefanPro </t>
+  </si>
+  <si>
+    <t>Einzelner MacOS Rechner, technicsher user novaadm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ggfs Anpassung für Terminal Profile, Software Build
+</t>
+  </si>
+  <si>
+    <t>Prio</t>
+  </si>
+  <si>
+    <t>Postpone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Next </t>
+  </si>
+  <si>
+    <t>Starte auf Worker node i Workload mit Parameter</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -371,8 +514,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="22"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -403,8 +553,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="16">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -593,11 +755,49 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -614,93 +814,149 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1057,6 +1313,404 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4433BE9-E73B-BD48-83BD-771F1C1F09BA}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A2:G35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="23.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="46.6640625" customWidth="1"/>
+    <col min="3" max="3" width="26.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="46.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="3.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:7" ht="29" x14ac:dyDescent="0.2">
+      <c r="A2" s="33" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="49" t="s">
+        <v>89</v>
+      </c>
+      <c r="E2" s="49" t="s">
+        <v>99</v>
+      </c>
+      <c r="F2" s="48"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+    </row>
+    <row r="4" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="1"/>
+    </row>
+    <row r="5" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A5" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="G5" s="1"/>
+    </row>
+    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.2">
+      <c r="A6" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="D6" s="50" t="s">
+        <v>90</v>
+      </c>
+      <c r="E6" s="50"/>
+      <c r="G6" s="1"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="D7" s="50" t="s">
+        <v>90</v>
+      </c>
+      <c r="E7" s="50"/>
+      <c r="G7" s="1"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C8" s="14"/>
+      <c r="D8" s="50" t="s">
+        <v>90</v>
+      </c>
+      <c r="E8" s="50"/>
+      <c r="G8" s="1"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" s="53" t="s">
+        <v>91</v>
+      </c>
+      <c r="E9" s="53" t="s">
+        <v>100</v>
+      </c>
+      <c r="G9" s="1"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="D10" s="50" t="s">
+        <v>90</v>
+      </c>
+      <c r="E10" s="50"/>
+      <c r="G10" s="1"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C11" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="D11" s="51" t="s">
+        <v>92</v>
+      </c>
+      <c r="E11" s="51" t="s">
+        <v>101</v>
+      </c>
+      <c r="G11" s="1"/>
+    </row>
+    <row r="12" spans="1:7" ht="52" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="28" t="s">
+        <v>82</v>
+      </c>
+      <c r="B12" s="29" t="s">
+        <v>83</v>
+      </c>
+      <c r="C12" s="30"/>
+      <c r="D12" s="52" t="s">
+        <v>93</v>
+      </c>
+      <c r="E12" s="52" t="s">
+        <v>101</v>
+      </c>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+    </row>
+    <row r="13" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+    </row>
+    <row r="14" spans="1:7" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+    </row>
+    <row r="15" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A15" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="31" t="s">
+        <v>5</v>
+      </c>
+      <c r="C15" s="32" t="s">
+        <v>19</v>
+      </c>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+    </row>
+    <row r="16" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A16" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="D17" s="50" t="s">
+        <v>90</v>
+      </c>
+      <c r="E17" s="50"/>
+    </row>
+    <row r="18" spans="1:5" ht="68" x14ac:dyDescent="0.2">
+      <c r="A18" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="E18" s="50" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C19" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="D19" s="50"/>
+      <c r="E19" s="50"/>
+    </row>
+    <row r="20" spans="1:5" ht="60" x14ac:dyDescent="0.2">
+      <c r="A20" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C20" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="D20" s="50"/>
+      <c r="E20" s="50"/>
+    </row>
+    <row r="21" spans="1:5" ht="135" x14ac:dyDescent="0.2">
+      <c r="A21" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="E21" s="50" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="45" x14ac:dyDescent="0.2">
+      <c r="A22" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C22" s="14"/>
+      <c r="D22" s="50"/>
+      <c r="E22" s="50"/>
+    </row>
+    <row r="23" spans="1:5" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="B23" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="C23" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="D23" s="50"/>
+      <c r="E23" s="50"/>
+    </row>
+    <row r="25" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B25" s="23"/>
+      <c r="C25" s="23"/>
+    </row>
+    <row r="26" spans="1:5" ht="18" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B26" s="34" t="s">
+        <v>0</v>
+      </c>
+      <c r="C26" s="35" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="90" x14ac:dyDescent="0.2">
+      <c r="A27" s="38" t="s">
+        <v>30</v>
+      </c>
+      <c r="B27" s="39" t="s">
+        <v>79</v>
+      </c>
+      <c r="C27" s="40" t="s">
+        <v>80</v>
+      </c>
+      <c r="D27" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="75" x14ac:dyDescent="0.2">
+      <c r="A28" s="41" t="s">
+        <v>31</v>
+      </c>
+      <c r="B28" s="36" t="s">
+        <v>81</v>
+      </c>
+      <c r="C28" s="42" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="30" x14ac:dyDescent="0.2">
+      <c r="A29" s="43" t="s">
+        <v>70</v>
+      </c>
+      <c r="B29" s="37" t="s">
+        <v>71</v>
+      </c>
+      <c r="C29" s="44" t="s">
+        <v>72</v>
+      </c>
+      <c r="D29" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="91" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="45" t="s">
+        <v>85</v>
+      </c>
+      <c r="B30" s="46" t="s">
+        <v>102</v>
+      </c>
+      <c r="C30" s="47" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A35" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="76" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{376C7D14-C569-E842-B4FC-364E7F3B9A74}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -1074,11 +1728,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" ht="29" x14ac:dyDescent="0.2">
-      <c r="A2" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
+      <c r="A2" s="33" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D3" s="1"/>
@@ -1087,82 +1741,82 @@
       <c r="G3" s="1"/>
     </row>
     <row r="4" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="9" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="15" t="s">
-        <v>20</v>
+      <c r="C5" s="12" t="s">
+        <v>19</v>
       </c>
       <c r="G5" s="1"/>
     </row>
     <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.2">
-      <c r="A6" s="16" t="s">
-        <v>41</v>
+      <c r="A6" s="13" t="s">
+        <v>37</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C6" s="17" t="s">
-        <v>50</v>
+        <v>46</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>45</v>
       </c>
       <c r="G6" s="1"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="15" t="s">
         <v>2</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="19" t="s">
-        <v>27</v>
+      <c r="C7" s="16" t="s">
+        <v>26</v>
       </c>
       <c r="G7" s="1"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" s="20" t="s">
-        <v>46</v>
+      <c r="A8" s="17" t="s">
+        <v>41</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="C8" s="17" t="s">
         <v>47</v>
       </c>
+      <c r="C8" s="14" t="s">
+        <v>42</v>
+      </c>
       <c r="G8" s="1"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="18" t="s">
         <v>9</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="22" t="s">
+      <c r="C9" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="G9" s="1"/>
+    </row>
+    <row r="10" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="28" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" s="29" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="G9" s="1"/>
-    </row>
-    <row r="10" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="31" t="s">
-        <v>4</v>
-      </c>
-      <c r="B10" s="32" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" s="33" t="s">
-        <v>18</v>
-      </c>
-      <c r="D10" s="7"/>
+      <c r="D10" s="1"/>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
@@ -1174,25 +1828,25 @@
       <c r="G11" s="1"/>
     </row>
     <row r="12" spans="1:7" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
     </row>
     <row r="13" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A13" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" s="34" t="s">
+      <c r="A13" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="C13" s="35" t="s">
-        <v>20</v>
+      <c r="C13" s="32" t="s">
+        <v>19</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
@@ -1200,14 +1854,14 @@
       <c r="G13" s="1"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A14" s="16" t="s">
-        <v>23</v>
+      <c r="A14" s="13" t="s">
+        <v>22</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C14" s="17" t="s">
-        <v>16</v>
+        <v>44</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>15</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
@@ -1215,414 +1869,119 @@
       <c r="G14" s="1"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A15" s="18" t="s">
-        <v>21</v>
+      <c r="A15" s="15" t="s">
+        <v>20</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C15" s="19" t="s">
-        <v>19</v>
+        <v>34</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" s="20" t="s">
+      <c r="A16" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="C16" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="C16" s="17" t="s">
-        <v>26</v>
-      </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" s="21" t="s">
+      <c r="A17" s="18" t="s">
         <v>12</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C17" s="22" t="s">
-        <v>38</v>
+      <c r="C17" s="19" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" s="16" t="s">
+      <c r="A18" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C18" s="17" t="s">
+      <c r="B19" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19" s="16" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="45" x14ac:dyDescent="0.2">
+      <c r="A20" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="14"/>
+    </row>
+    <row r="21" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="22" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="C21" s="21" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C19" s="19" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="45" x14ac:dyDescent="0.2">
-      <c r="A20" s="20" t="s">
+    <row r="23" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B23" s="23"/>
+      <c r="C23" s="23"/>
+    </row>
+    <row r="24" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A24" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B24" s="24" t="s">
+        <v>0</v>
+      </c>
+      <c r="C24" s="25" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="180" x14ac:dyDescent="0.2">
+      <c r="A25" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="B20" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C20" s="17"/>
-    </row>
-    <row r="21" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="25" t="s">
-        <v>24</v>
-      </c>
-      <c r="B21" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="C21" s="24" t="s">
+      <c r="B25" s="8" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B23" s="26"/>
-      <c r="C23" s="26"/>
-    </row>
-    <row r="24" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A24" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="B24" s="27" t="s">
-        <v>0</v>
-      </c>
-      <c r="C24" s="28" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="180" x14ac:dyDescent="0.2">
-      <c r="A25" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="B25" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="C25" s="29" t="s">
-        <v>57</v>
+      <c r="C25" s="26" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="61" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="30" t="s">
-        <v>33</v>
-      </c>
-      <c r="B26" s="23" t="s">
-        <v>54</v>
-      </c>
-      <c r="C26" s="24" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A27" s="11"/>
-      <c r="B27" s="11"/>
-      <c r="C27" s="11"/>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A33" s="2"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:C2"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="76" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09BF5F13-9A9E-7B47-A5AE-CA19DB2EFF62}">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A2:G33"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="23.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="46.6640625" customWidth="1"/>
-    <col min="3" max="3" width="26.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.6640625" customWidth="1"/>
-    <col min="5" max="5" width="46.6640625" customWidth="1"/>
-    <col min="6" max="6" width="25" customWidth="1"/>
-    <col min="7" max="7" width="3.6640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="1:7" ht="29" x14ac:dyDescent="0.2">
-      <c r="A2" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-    </row>
-    <row r="4" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="1"/>
-    </row>
-    <row r="5" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A5" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="G5" s="1"/>
-    </row>
-    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.2">
-      <c r="A6" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C6" s="17" t="s">
+      <c r="A26" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B26" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="C26" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="G6" s="1"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" s="18" t="s">
-        <v>2</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="G7" s="1"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" s="20" t="s">
-        <v>46</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="C8" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="G8" s="1"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" s="21" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" s="22" t="s">
-        <v>17</v>
-      </c>
-      <c r="G9" s="1"/>
-    </row>
-    <row r="10" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="31" t="s">
-        <v>4</v>
-      </c>
-      <c r="B10" s="32" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" s="33" t="s">
-        <v>18</v>
-      </c>
-      <c r="D10" s="7"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-    </row>
-    <row r="11" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-    </row>
-    <row r="12" spans="1:7" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
-    </row>
-    <row r="13" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A13" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" s="34" t="s">
-        <v>5</v>
-      </c>
-      <c r="C13" s="35" t="s">
-        <v>20</v>
-      </c>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A14" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C14" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A15" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C15" s="19" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" s="20" t="s">
-        <v>24</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C16" s="17" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C17" s="22" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C18" s="17" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C19" s="19" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.2">
-      <c r="A20" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C20" s="17"/>
-    </row>
-    <row r="21" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="25" t="s">
-        <v>24</v>
-      </c>
-      <c r="B21" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="C21" s="24" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B23" s="26"/>
-      <c r="C23" s="26"/>
-    </row>
-    <row r="24" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A24" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="B24" s="27" t="s">
-        <v>0</v>
-      </c>
-      <c r="C24" s="28" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="195" x14ac:dyDescent="0.2">
-      <c r="A25" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="B25" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="C25" s="29" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="61" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="30" t="s">
-        <v>33</v>
-      </c>
-      <c r="B26" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="C26" s="24" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A27" s="11"/>
-      <c r="B27" s="11"/>
-      <c r="C27" s="11"/>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A33" s="2"/>

</xml_diff>

<commit_message>
doc : added Scenario to runbook
</commit_message>
<xml_diff>
--- a/docs/nova_overview.xlsx
+++ b/docs/nova_overview.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stefan_pro/Documents/Claude/Projects/nova/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{0130EE51-885D-AF44-9BA1-90AFB7AC42E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{43743682-9B96-2746-B08C-05C19919028C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="38400" windowHeight="24980" activeTab="5" xr2:uid="{189BD8D0-FCFC-8748-8061-DE49C9010CB9}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="241">
   <si>
     <t>Zielsetzung</t>
   </si>
@@ -802,12 +802,291 @@
   <si>
     <t>~/nova/scripts/nova_run.sh lab_ingest_fx nova-hub --params-file ~/jobs/lab_ingest_fx_daily.json</t>
   </si>
+  <si>
+    <t>sudo ~/nova/scripts/install_lab_ingest_fx_daemon.sh</t>
+  </si>
+  <si>
+    <t>ssh nova-w5 ~/nova/scripts/node_deploy.sh</t>
+  </si>
+  <si>
+    <t>Szenario Analyse</t>
+  </si>
+  <si>
+    <t>cat &gt; ~/scenarios/tech_crash_2026.json &lt;&lt;'EOF'
+{
+  "name": "Tech crash + USD weakness 2026",
+  "shocks": [
+    {"target": "asset_class", "value": "stock", "pct": -15},
+    {"target": "symbol",      "value": "NVDA",  "pct": -40},
+    {"target": "symbol",      "value": "AAPL",  "pct": -25},
+    {"target": "currency",    "value": "USD",   "pct": -8}
+  ]
+}
+EOF</t>
+  </si>
+  <si>
+    <t>Szenario Liste</t>
+  </si>
+  <si>
+    <t>~/nova/workloads/lab_scenarios/run.sh list</t>
+  </si>
+  <si>
+    <t>select * from ref_scenarios;
+select * from ref_scenario_shocks;</t>
+  </si>
+  <si>
+    <t>duckDB</t>
+  </si>
+  <si>
+    <t>Szenario erstellen</t>
+  </si>
+  <si>
+    <t>script</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> JSON imput</t>
+  </si>
+  <si>
+    <r>
+      <t>~/nova/workloads/</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>lab</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>_</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>scenarios</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">/run.sh </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>save</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> tech_crash_2026 ~/scenarios/tech_crash_2026.json --tags "stress,tech,2026"</t>
+    </r>
+  </si>
+  <si>
+    <t>Szenario Run</t>
+  </si>
+  <si>
+    <r>
+      <t>~/nova/workloads/</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>lab_scenarios</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">/run.sh </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>run-saved</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> tech_crash_2026 --top </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF008080"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>10</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>/nova/workloads/</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>lab_scenarios</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">/run.sh </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>show</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> tech_crash_2026</t>
+    </r>
+  </si>
+  <si>
+    <t>ad-hoc JSON</t>
+  </si>
+  <si>
+    <r>
+      <t>~/nova/workloads/</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>lab_scenarios</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>/run.sh run ~/scenarios/soft_landing.json --top 15</t>
+    </r>
+  </si>
+  <si>
+    <t>gespeichert in ref_scenarios</t>
+  </si>
+  <si>
+    <t>select * from sig_scenario_runs;</t>
+  </si>
+  <si>
+    <t>scripts</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">~/nova/workloads/lab_scenarios/run.sh </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Textkörper)"/>
+      </rPr>
+      <t>history</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> tech_crash_2026</t>
+    </r>
+  </si>
+  <si>
+    <t>Szenario , Details zu Lauf</t>
+  </si>
+  <si>
+    <t>Szenario, Historie</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20">
+  <fonts count="22">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -945,6 +1224,19 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF008080"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow (Textkörper)"/>
     </font>
   </fonts>
   <fills count="12">
@@ -1246,7 +1538,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1451,6 +1743,15 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="10" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3154,7 +3455,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B24AAE9F-B375-5A4A-8E8D-2A7896F640DD}">
-  <dimension ref="A1:D53"/>
+  <dimension ref="A1:D73"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="43.6640625" customWidth="1"/>
@@ -3191,11 +3492,13 @@
         <v>113</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" ht="17">
       <c r="A3" s="67"/>
       <c r="B3" s="67"/>
       <c r="C3" s="68"/>
-      <c r="D3" s="69"/>
+      <c r="D3" s="69" t="s">
+        <v>219</v>
+      </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="67"/>
@@ -3327,35 +3630,37 @@
       <c r="A20" s="66"/>
       <c r="B20" s="67"/>
       <c r="C20" s="68"/>
-      <c r="D20" s="69"/>
-    </row>
-    <row r="21" spans="1:4" ht="17">
+      <c r="D20" s="69" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
       <c r="A21" s="66"/>
-      <c r="B21" s="67" t="s">
-        <v>208</v>
-      </c>
-      <c r="C21" s="68" t="s">
-        <v>209</v>
-      </c>
-      <c r="D21" s="69" t="s">
-        <v>210</v>
-      </c>
+      <c r="B21" s="67"/>
+      <c r="C21" s="68"/>
+      <c r="D21" s="69"/>
     </row>
     <row r="22" spans="1:4" ht="17">
       <c r="A22" s="66"/>
-      <c r="B22" s="67"/>
+      <c r="B22" s="67" t="s">
+        <v>208</v>
+      </c>
       <c r="C22" s="68" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D22" s="69" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="17">
       <c r="A23" s="66"/>
       <c r="B23" s="67"/>
-      <c r="C23" s="68"/>
-      <c r="D23" s="69"/>
+      <c r="C23" s="68" t="s">
+        <v>211</v>
+      </c>
+      <c r="D23" s="69" t="s">
+        <v>212</v>
+      </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="66"/>
@@ -3365,136 +3670,136 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="66"/>
-      <c r="B25" s="67" t="s">
+      <c r="B25" s="67"/>
+      <c r="C25" s="68"/>
+      <c r="D25" s="69"/>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" s="66"/>
+      <c r="B26" s="67" t="s">
         <v>213</v>
       </c>
-      <c r="C25" s="68"/>
-      <c r="D25" s="69" t="s">
+      <c r="C26" s="68"/>
+      <c r="D26" s="69" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
-      <c r="A26" s="67"/>
-      <c r="B26" s="67"/>
-      <c r="C26" s="68"/>
-      <c r="D26" s="69"/>
-    </row>
-    <row r="27" spans="1:4" ht="17">
-      <c r="A27" s="58" t="s">
+    <row r="27" spans="1:4">
+      <c r="A27" s="67"/>
+      <c r="B27" s="67"/>
+      <c r="C27" s="68"/>
+      <c r="D27" s="69"/>
+    </row>
+    <row r="28" spans="1:4" ht="17">
+      <c r="A28" s="58" t="s">
         <v>166</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B28" t="s">
         <v>194</v>
-      </c>
-      <c r="C27" s="60"/>
-      <c r="D27" s="65" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="17">
-      <c r="B28" t="s">
-        <v>167</v>
       </c>
       <c r="C28" s="60"/>
       <c r="D28" s="65" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="17">
+      <c r="B29" t="s">
+        <v>167</v>
+      </c>
       <c r="C29" s="60"/>
       <c r="D29" s="65" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="17">
+      <c r="C30" s="60"/>
+      <c r="D30" s="65" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="17">
-      <c r="B30" t="s">
+    <row r="31" spans="1:4" ht="17">
+      <c r="B31" t="s">
         <v>171</v>
       </c>
-      <c r="C30" s="60"/>
-      <c r="D30" s="71" t="s">
+      <c r="C31" s="60"/>
+      <c r="D31" s="71" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="17">
-      <c r="C31" s="60"/>
-      <c r="D31" s="65" t="s">
+    <row r="32" spans="1:4" ht="17">
+      <c r="C32" s="60"/>
+      <c r="D32" s="65" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="32" spans="1:4">
-      <c r="C32" s="60"/>
-      <c r="D32" s="65"/>
-    </row>
-    <row r="33" spans="1:4" ht="51">
-      <c r="B33" t="s">
+    <row r="33" spans="1:4">
+      <c r="C33" s="60"/>
+      <c r="D33" s="65"/>
+    </row>
+    <row r="34" spans="1:4" ht="51">
+      <c r="B34" t="s">
         <v>188</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C34" t="s">
         <v>187</v>
       </c>
-      <c r="D33" s="53" t="s">
+      <c r="D34" s="53" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="51">
-      <c r="D34" s="53" t="s">
+    <row r="35" spans="1:4" ht="51">
+      <c r="D35" s="53" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="51">
-      <c r="B37" t="s">
+    <row r="38" spans="1:4" ht="51">
+      <c r="B38" t="s">
         <v>189</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C38" t="s">
         <v>187</v>
       </c>
-      <c r="D37" s="53" t="s">
+      <c r="D38" s="53" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="40" spans="1:4">
-      <c r="A40" s="66" t="s">
+    <row r="41" spans="1:4">
+      <c r="A41" s="66" t="s">
         <v>75</v>
       </c>
-      <c r="B40" s="67" t="s">
+      <c r="B41" s="67" t="s">
         <v>164</v>
       </c>
-      <c r="C40" s="68" t="s">
+      <c r="C41" s="68" t="s">
         <v>165</v>
       </c>
-      <c r="D40" s="70" t="s">
+      <c r="D41" s="70" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="41" spans="1:4" ht="17">
-      <c r="A41" s="67"/>
-      <c r="B41" s="67"/>
-      <c r="C41" s="67"/>
-      <c r="D41" s="70" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4">
+    <row r="42" spans="1:4" ht="17">
       <c r="A42" s="67"/>
       <c r="B42" s="67"/>
       <c r="C42" s="67"/>
-      <c r="D42" s="70"/>
-    </row>
-    <row r="43" spans="1:4" ht="17">
+      <c r="D42" s="70" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
       <c r="A43" s="67"/>
       <c r="B43" s="67"/>
-      <c r="C43" s="67" t="s">
-        <v>196</v>
-      </c>
-      <c r="D43" s="70" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4">
+      <c r="C43" s="67"/>
+      <c r="D43" s="70"/>
+    </row>
+    <row r="44" spans="1:4" ht="17">
       <c r="A44" s="67"/>
       <c r="B44" s="67"/>
-      <c r="C44" s="67"/>
-      <c r="D44" s="70"/>
+      <c r="C44" s="67" t="s">
+        <v>196</v>
+      </c>
+      <c r="D44" s="70" t="s">
+        <v>199</v>
+      </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="67"/>
@@ -3506,53 +3811,197 @@
       <c r="A46" s="67"/>
       <c r="B46" s="67"/>
       <c r="C46" s="67"/>
-      <c r="D46" s="69"/>
+      <c r="D46" s="70"/>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="67"/>
       <c r="B47" s="67"/>
       <c r="C47" s="67"/>
-      <c r="D47" s="70"/>
-    </row>
-    <row r="48" spans="1:4" ht="17">
+      <c r="D47" s="69"/>
+    </row>
+    <row r="48" spans="1:4">
       <c r="A48" s="67"/>
       <c r="B48" s="67"/>
-      <c r="C48" s="67" t="s">
-        <v>200</v>
-      </c>
-      <c r="D48" s="70" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4">
+      <c r="C48" s="67"/>
+      <c r="D48" s="70"/>
+    </row>
+    <row r="49" spans="1:4" ht="17">
       <c r="A49" s="67"/>
       <c r="B49" s="67"/>
-      <c r="C49" s="67"/>
-      <c r="D49" s="70"/>
+      <c r="C49" s="67" t="s">
+        <v>200</v>
+      </c>
+      <c r="D49" s="70" t="s">
+        <v>201</v>
+      </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="67"/>
       <c r="B50" s="67"/>
-      <c r="C50" s="67" t="s">
-        <v>203</v>
-      </c>
-      <c r="D50" t="s">
-        <v>202</v>
-      </c>
+      <c r="C50" s="67"/>
+      <c r="D50" s="70"/>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="67"/>
       <c r="B51" s="67"/>
-      <c r="C51" s="67"/>
-      <c r="D51" s="70"/>
-    </row>
-    <row r="53" spans="1:4">
-      <c r="C53" t="s">
+      <c r="C51" s="67" t="s">
+        <v>203</v>
+      </c>
+      <c r="D51" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4">
+      <c r="A52" s="67"/>
+      <c r="B52" s="67"/>
+      <c r="C52" s="67"/>
+      <c r="D52" s="70"/>
+    </row>
+    <row r="54" spans="1:4">
+      <c r="C54" t="s">
         <v>216</v>
       </c>
-      <c r="D53" s="53" t="s">
+      <c r="D54" s="53" t="s">
         <v>217</v>
       </c>
+    </row>
+    <row r="59" spans="1:4" ht="113" customHeight="1">
+      <c r="A59" s="66" t="s">
+        <v>220</v>
+      </c>
+      <c r="B59" s="77" t="s">
+        <v>226</v>
+      </c>
+      <c r="C59" s="77" t="s">
+        <v>228</v>
+      </c>
+      <c r="D59" s="70" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="17">
+      <c r="A60" s="67"/>
+      <c r="B60" s="67"/>
+      <c r="C60" s="67" t="s">
+        <v>227</v>
+      </c>
+      <c r="D60" s="70" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
+      <c r="A61" s="67"/>
+      <c r="B61" s="67"/>
+      <c r="C61" s="67"/>
+      <c r="D61" s="70"/>
+    </row>
+    <row r="62" spans="1:4">
+      <c r="A62" s="67"/>
+      <c r="B62" s="67" t="s">
+        <v>222</v>
+      </c>
+      <c r="C62" s="67" t="s">
+        <v>237</v>
+      </c>
+      <c r="D62" s="67" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" ht="34">
+      <c r="A63" s="67"/>
+      <c r="B63" s="67"/>
+      <c r="C63" s="76" t="s">
+        <v>225</v>
+      </c>
+      <c r="D63" s="75" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4">
+      <c r="A64" s="67"/>
+      <c r="B64" s="67"/>
+      <c r="C64" s="67"/>
+      <c r="D64" s="70"/>
+    </row>
+    <row r="65" spans="1:4">
+      <c r="A65" s="67"/>
+      <c r="B65" s="67" t="s">
+        <v>230</v>
+      </c>
+      <c r="C65" s="67" t="s">
+        <v>233</v>
+      </c>
+      <c r="D65" s="67" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4">
+      <c r="A66" s="67"/>
+      <c r="B66" s="67"/>
+      <c r="C66" s="67" t="s">
+        <v>235</v>
+      </c>
+      <c r="D66" s="67" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4">
+      <c r="A67" s="67"/>
+      <c r="B67" s="67"/>
+      <c r="C67" s="67"/>
+      <c r="D67" s="70"/>
+    </row>
+    <row r="68" spans="1:4">
+      <c r="A68" s="67"/>
+      <c r="B68" s="67" t="s">
+        <v>239</v>
+      </c>
+      <c r="C68" s="67" t="s">
+        <v>227</v>
+      </c>
+      <c r="D68" s="67" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4">
+      <c r="A69" s="67"/>
+      <c r="B69" s="67"/>
+      <c r="C69" s="67" t="s">
+        <v>225</v>
+      </c>
+      <c r="D69" s="70" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4">
+      <c r="A70" s="67"/>
+      <c r="B70" s="67"/>
+      <c r="C70" s="67"/>
+      <c r="D70" s="70"/>
+    </row>
+    <row r="71" spans="1:4">
+      <c r="A71" s="67"/>
+      <c r="B71" s="67" t="s">
+        <v>240</v>
+      </c>
+      <c r="C71" s="67"/>
+      <c r="D71" s="67" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" ht="17">
+      <c r="A72" s="67"/>
+      <c r="B72" s="67"/>
+      <c r="C72" s="67"/>
+      <c r="D72" s="70" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4">
+      <c r="A73" s="67"/>
+      <c r="B73" s="67"/>
+      <c r="C73" s="67"/>
+      <c r="D73" s="70"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
doc: added alias section
</commit_message>
<xml_diff>
--- a/docs/nova_overview.xlsx
+++ b/docs/nova_overview.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stefan_pro/Documents/Claude/Projects/nova/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{43743682-9B96-2746-B08C-05C19919028C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{C1AF726C-B524-0C4A-A192-61FBA343E713}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="38400" windowHeight="24980" activeTab="5" xr2:uid="{189BD8D0-FCFC-8748-8061-DE49C9010CB9}"/>
   </bookViews>
@@ -19,6 +19,9 @@
     <sheet name="V1" sheetId="2" r:id="rId4"/>
     <sheet name="Utilities" sheetId="5" r:id="rId5"/>
     <sheet name="Runbook" sheetId="6" r:id="rId6"/>
+    <sheet name="Szenario_Analyse" sheetId="8" r:id="rId7"/>
+    <sheet name="Historical Replay" sheetId="9" r:id="rId8"/>
+    <sheet name="alias" sheetId="11" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Planning!$A$2:$C$50</definedName>
@@ -47,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="274">
   <si>
     <t>Zielsetzung</t>
   </si>
@@ -1081,12 +1084,354 @@
   <si>
     <t>Szenario, Historie</t>
   </si>
+  <si>
+    <t>Architektur</t>
+  </si>
+  <si>
+    <r>
+      <t>Mathematik:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> für jeden historischen Tag </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>t</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> im Lookback-Window:</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">pro Holding: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>value_t = quantity × close_at_t × fx_to_base_at_t</t>
+    </r>
+  </si>
+  <si>
+    <t>Portfolio-Total = SUM across holdings</t>
+  </si>
+  <si>
+    <t>Day-over-day deltas, rolling 5-day windows, running-peak-drawdown</t>
+  </si>
+  <si>
+    <t>Subcommands:</t>
+  </si>
+  <si>
+    <r>
+      <t>worst-day [--lookback-days 730] [--top 10]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — N schlimmste Einzeltage</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>worst-week [--lookback-days 730] [--top 10]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — N schlimmste 5-Trading-Day-Windows</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>drawdown [--lookback-days 730]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — Maximum-Drawdown peak→trough</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>replay --from YYYY-MM-DD --to YYYY-MM-DD [--csv]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — Tag-für-Tag Time-Series</t>
+    </r>
+  </si>
+  <si>
+    <t># 1. Was war der schlimmste Tag in den letzten 2 Jahren mit deinem heutigen Portfolio?</t>
+  </si>
+  <si>
+    <t>~/nova/workloads/lab_replay/run.sh worst-day --top 10</t>
+  </si>
+  <si>
+    <t># 2. Schlimmste 5-Trading-Day-Windows (entspricht ~1 Woche)</t>
+  </si>
+  <si>
+    <t>~/nova/workloads/lab_replay/run.sh worst-week --top 5</t>
+  </si>
+  <si>
+    <t># 3. Maximum Drawdown — peak-to-trough Analyse</t>
+  </si>
+  <si>
+    <t>~/nova/workloads/lab_replay/run.sh drawdown</t>
+  </si>
+  <si>
+    <t># 4. Full Replay über bestimmten Zeitraum (z.B. 2024 Q4)</t>
+  </si>
+  <si>
+    <t>~/nova/workloads/lab_replay/run.sh replay --from 2024-10-01 --to 2024-12-31 --csv</t>
+  </si>
+  <si>
+    <t># 5. Aggressivere Settings — schau ueber den ganzen Mai-2024-bis-jetzt Zeitraum</t>
+  </si>
+  <si>
+    <t>~/nova/workloads/lab_replay/run.sh worst-day --lookback-days 365 --top 20</t>
+  </si>
+  <si>
+    <t>~/nova/workloads/lab_replay/run.sh drawdown --lookback-days 365</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">alias </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Textkörper)"/>
+      </rPr>
+      <t>db</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>='duckdb ~/nova_data/lab.duckdb'</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">alias </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>nova_db</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>=~/nova/nova_db.sh</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">alias </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ns</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>=~/nova/scripts/nova_status.sh</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">alias </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>logs</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>='ll ~/nova_jobs/logs'</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">alias </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>jobs</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>='ll ~/nova_jobs'</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">alias </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>viewlog</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>='less $(ls -t ~/nova_jobs/logs/*.log | head -n 1)'</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">alias </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>taillog</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>='tail -f  $(ls -t ~/nova_jobs/logs/*.log | head -n 1)'</t>
+    </r>
+  </si>
+  <si>
+    <t>alias nova='cd ~/nova'</t>
+  </si>
+  <si>
+    <t>alias nova-lab='cd ~/nova-lab'</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> alias nd='~/nova/scripts/node_deploy.sh'</t>
+  </si>
+  <si>
+    <t>CSP</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> sudo launchctl kickstart system/de.gershu.nova.lab.screener_csp</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22">
+  <fonts count="26">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1226,6 +1571,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="12"/>
       <color rgb="FF008080"/>
       <name val="Aptos Narrow"/>
@@ -1235,6 +1588,26 @@
     <font>
       <b/>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow (Textkörper)"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13.5"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
       <color theme="1"/>
       <name val="Aptos Narrow (Textkörper)"/>
     </font>
@@ -1538,7 +1911,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1753,6 +2126,9 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -3455,7 +3831,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B24AAE9F-B375-5A4A-8E8D-2A7896F640DD}">
-  <dimension ref="A1:D73"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="43.6640625" customWidth="1"/>
@@ -3865,143 +4241,355 @@
         <v>217</v>
       </c>
     </row>
-    <row r="59" spans="1:4" ht="113" customHeight="1">
-      <c r="A59" s="66" t="s">
+    <row r="56" spans="1:4">
+      <c r="C56" t="s">
+        <v>272</v>
+      </c>
+      <c r="D56" s="53" t="s">
+        <v>273</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7326FA95-29FD-5D48-800E-46AF885A176A}">
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="44.6640625" defaultRowHeight="16"/>
+  <cols>
+    <col min="4" max="4" width="68.83203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="187">
+      <c r="A1" s="66" t="s">
         <v>220</v>
       </c>
-      <c r="B59" s="77" t="s">
+      <c r="B1" s="77" t="s">
         <v>226</v>
       </c>
-      <c r="C59" s="77" t="s">
+      <c r="C1" s="77" t="s">
         <v>228</v>
       </c>
-      <c r="D59" s="70" t="s">
+      <c r="D1" s="70" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="60" spans="1:4" ht="17">
-      <c r="A60" s="67"/>
-      <c r="B60" s="67"/>
-      <c r="C60" s="67" t="s">
+    <row r="2" spans="1:4" ht="34">
+      <c r="A2" s="67"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67" t="s">
         <v>227</v>
       </c>
-      <c r="D60" s="70" t="s">
+      <c r="D2" s="70" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="61" spans="1:4">
-      <c r="A61" s="67"/>
-      <c r="B61" s="67"/>
-      <c r="C61" s="67"/>
-      <c r="D61" s="70"/>
-    </row>
-    <row r="62" spans="1:4">
-      <c r="A62" s="67"/>
-      <c r="B62" s="67" t="s">
+    <row r="3" spans="1:4">
+      <c r="A3" s="67"/>
+      <c r="B3" s="67"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="70"/>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="67"/>
+      <c r="B4" s="67" t="s">
         <v>222</v>
       </c>
-      <c r="C62" s="67" t="s">
+      <c r="C4" s="67" t="s">
         <v>237</v>
       </c>
-      <c r="D62" s="67" t="s">
+      <c r="D4" s="67" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="63" spans="1:4" ht="34">
-      <c r="A63" s="67"/>
-      <c r="B63" s="67"/>
-      <c r="C63" s="76" t="s">
+    <row r="5" spans="1:4" ht="34">
+      <c r="A5" s="67"/>
+      <c r="B5" s="67"/>
+      <c r="C5" s="76" t="s">
         <v>225</v>
       </c>
-      <c r="D63" s="75" t="s">
+      <c r="D5" s="75" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="64" spans="1:4">
-      <c r="A64" s="67"/>
-      <c r="B64" s="67"/>
-      <c r="C64" s="67"/>
-      <c r="D64" s="70"/>
-    </row>
-    <row r="65" spans="1:4">
-      <c r="A65" s="67"/>
-      <c r="B65" s="67" t="s">
+    <row r="6" spans="1:4">
+      <c r="A6" s="67"/>
+      <c r="B6" s="67"/>
+      <c r="C6" s="67"/>
+      <c r="D6" s="70"/>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="67"/>
+      <c r="B7" s="67" t="s">
         <v>230</v>
       </c>
-      <c r="C65" s="67" t="s">
+      <c r="C7" s="67" t="s">
         <v>233</v>
       </c>
-      <c r="D65" s="67" t="s">
+      <c r="D7" s="67" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="66" spans="1:4">
-      <c r="A66" s="67"/>
-      <c r="B66" s="67"/>
-      <c r="C66" s="67" t="s">
+    <row r="8" spans="1:4">
+      <c r="A8" s="67"/>
+      <c r="B8" s="67"/>
+      <c r="C8" s="67" t="s">
         <v>235</v>
       </c>
-      <c r="D66" s="67" t="s">
+      <c r="D8" s="67" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="67" spans="1:4">
-      <c r="A67" s="67"/>
-      <c r="B67" s="67"/>
-      <c r="C67" s="67"/>
-      <c r="D67" s="70"/>
-    </row>
-    <row r="68" spans="1:4">
-      <c r="A68" s="67"/>
-      <c r="B68" s="67" t="s">
+    <row r="9" spans="1:4">
+      <c r="A9" s="67"/>
+      <c r="B9" s="67"/>
+      <c r="C9" s="67"/>
+      <c r="D9" s="70"/>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="67"/>
+      <c r="B10" s="67" t="s">
         <v>239</v>
       </c>
-      <c r="C68" s="67" t="s">
+      <c r="C10" s="67" t="s">
         <v>227</v>
       </c>
-      <c r="D68" s="67" t="s">
+      <c r="D10" s="67" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="69" spans="1:4">
-      <c r="A69" s="67"/>
-      <c r="B69" s="67"/>
-      <c r="C69" s="67" t="s">
+    <row r="11" spans="1:4" ht="17">
+      <c r="A11" s="67"/>
+      <c r="B11" s="67"/>
+      <c r="C11" s="67" t="s">
         <v>225</v>
       </c>
-      <c r="D69" s="70" t="s">
+      <c r="D11" s="70" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="70" spans="1:4">
-      <c r="A70" s="67"/>
-      <c r="B70" s="67"/>
-      <c r="C70" s="67"/>
-      <c r="D70" s="70"/>
-    </row>
-    <row r="71" spans="1:4">
-      <c r="A71" s="67"/>
-      <c r="B71" s="67" t="s">
+    <row r="12" spans="1:4">
+      <c r="A12" s="67"/>
+      <c r="B12" s="67"/>
+      <c r="C12" s="67"/>
+      <c r="D12" s="70"/>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" s="67"/>
+      <c r="B13" s="67" t="s">
         <v>240</v>
       </c>
-      <c r="C71" s="67"/>
-      <c r="D71" s="67" t="s">
+      <c r="C13" s="67"/>
+      <c r="D13" s="67" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="72" spans="1:4" ht="17">
-      <c r="A72" s="67"/>
-      <c r="B72" s="67"/>
-      <c r="C72" s="67"/>
-      <c r="D72" s="70" t="s">
+    <row r="14" spans="1:4" ht="17">
+      <c r="A14" s="67"/>
+      <c r="B14" s="67"/>
+      <c r="C14" s="67"/>
+      <c r="D14" s="70" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="73" spans="1:4">
-      <c r="A73" s="67"/>
-      <c r="B73" s="67"/>
-      <c r="C73" s="67"/>
-      <c r="D73" s="70"/>
+    <row r="15" spans="1:4">
+      <c r="A15" s="67"/>
+      <c r="B15" s="67"/>
+      <c r="C15" s="67"/>
+      <c r="D15" s="70"/>
+    </row>
+  </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6413202A-0FB5-304A-88E2-11392CE21654}">
+  <dimension ref="A1:E36"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col min="1" max="1" width="47.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="68.83203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="19">
+      <c r="A1" s="78" t="s">
+        <v>241</v>
+      </c>
+      <c r="E1" s="75"/>
+    </row>
+    <row r="3" spans="1:5" ht="17">
+      <c r="A3" s="79" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="17">
+      <c r="A5" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="79" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="17">
+      <c r="A11" s="80" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="17">
+      <c r="A12" s="80" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="17">
+      <c r="A13" s="80" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="17">
+      <c r="A14" s="80" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1">
+      <c r="A22" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1">
+      <c r="A23" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1">
+      <c r="A25" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1">
+      <c r="A26" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1">
+      <c r="A28" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1">
+      <c r="A29" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1">
+      <c r="A31" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1">
+      <c r="A32" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1">
+      <c r="A34" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1">
+      <c r="A35" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1">
+      <c r="A36" t="s">
+        <v>261</v>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19CA0FBA-888C-BE45-ACC4-14E7FF96C805}">
+  <dimension ref="A1:A10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetData>
+    <row r="1" spans="1:1" ht="22">
+      <c r="A1" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1">
+      <c r="A10" t="s">
+        <v>271</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>